<commit_message>
se anexan archivos de especificaciones
</commit_message>
<xml_diff>
--- a/Insumos/Entrada/DIRECTORIO NACIONAL (9).xlsx
+++ b/Insumos/Entrada/DIRECTORIO NACIONAL (9).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bancowcomco.sharepoint.com/sites/intranet/vp_tecnologia_operaciones/gr_operaciones/jfd_red_Agencias/Documentos_Publicos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PedrazaJh\Proyectos\Banco w\2026_INSENTIVOS_BANCO_W\Insumos\Entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8975" documentId="8_{24FF37B2-2879-40B7-8439-F557A2CFC6AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{253384B9-5AB4-4917-A80C-8AC864CE010F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B708F5-9BAD-44C0-8E4A-470905A343EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="3" state="hidden" r:id="rId1"/>
@@ -30,7 +30,7 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="18" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2266,7 +2266,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="51">
+  <fills count="52">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2543,6 +2543,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -3054,7 +3060,7 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" pivotButton="1" applyBorder="1"/>
@@ -3349,6 +3355,9 @@
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="33" fillId="51" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="236">
     <cellStyle name="20% - Énfasis1 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -3591,6 +3600,16 @@
   <dxfs count="10">
     <dxf>
       <font>
+        <color indexed="20"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor indexed="45"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3636,16 +3655,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="20"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="45"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5687,7 +5696,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Tabla dinámica1" cacheId="18" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Datos" updatedVersion="5" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Tabla dinámica1" cacheId="0" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Datos" updatedVersion="5" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
   <location ref="A3:B89" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
@@ -6353,11 +6362,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:B89"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="43.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="256" width="11.42578125" customWidth="1"/>
+    <col min="1" max="1" width="43.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="256" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:2">
@@ -7063,28 +7072,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:O141"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="12" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" style="54" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" style="55" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" style="55" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.5703125" style="13" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" style="13" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" style="54" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" style="55" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.453125" style="55" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.54296875" style="13" customWidth="1"/>
     <col min="6" max="6" width="44" style="13" customWidth="1"/>
-    <col min="7" max="7" width="41.42578125" style="13" customWidth="1"/>
-    <col min="8" max="8" width="36.140625" style="13" customWidth="1"/>
-    <col min="9" max="11" width="36.140625" style="9" customWidth="1"/>
-    <col min="12" max="12" width="52.42578125" style="13" customWidth="1"/>
-    <col min="13" max="13" width="61.140625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="41.453125" style="13" customWidth="1"/>
+    <col min="8" max="8" width="36.1796875" style="13" customWidth="1"/>
+    <col min="9" max="11" width="36.1796875" style="9" customWidth="1"/>
+    <col min="12" max="12" width="52.453125" style="13" customWidth="1"/>
+    <col min="13" max="13" width="61.1796875" style="13" customWidth="1"/>
     <col min="14" max="14" width="37" style="13" customWidth="1"/>
-    <col min="15" max="16384" width="11.42578125" style="13"/>
+    <col min="15" max="16384" width="11.453125" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="56" customFormat="1" ht="42.75" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="86" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="86" t="s">
         <v>89</v>
       </c>
       <c r="C1" s="63" t="s">
@@ -7124,7 +7133,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:14" s="9" customFormat="1" ht="23.25">
+    <row r="2" spans="1:14" s="9" customFormat="1" ht="23">
       <c r="A2" s="10" t="s">
         <v>102</v>
       </c>
@@ -7210,7 +7219,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="22.5">
+    <row r="4" spans="1:14" ht="23">
       <c r="A4" s="10" t="s">
         <v>103</v>
       </c>
@@ -7252,7 +7261,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="22.5">
+    <row r="5" spans="1:14" ht="23">
       <c r="A5" s="10" t="s">
         <v>121</v>
       </c>
@@ -7336,7 +7345,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="22.5">
+    <row r="7" spans="1:14" ht="23">
       <c r="A7" s="10" t="s">
         <v>130</v>
       </c>
@@ -7378,7 +7387,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="22.5">
+    <row r="8" spans="1:14" ht="23">
       <c r="A8" s="10" t="s">
         <v>133</v>
       </c>
@@ -7420,7 +7429,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="15">
+    <row r="9" spans="1:14" ht="14.5">
       <c r="A9" s="10" t="s">
         <v>136</v>
       </c>
@@ -7500,7 +7509,7 @@
       </c>
       <c r="N10" s="10"/>
     </row>
-    <row r="11" spans="1:14" ht="15">
+    <row r="11" spans="1:14" ht="14.5">
       <c r="A11" s="10" t="s">
         <v>145</v>
       </c>
@@ -7542,7 +7551,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="15">
+    <row r="12" spans="1:14" ht="14.5">
       <c r="A12" s="10" t="s">
         <v>149</v>
       </c>
@@ -7584,7 +7593,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="23.25">
+    <row r="13" spans="1:14" ht="23">
       <c r="A13" s="10" t="s">
         <v>153</v>
       </c>
@@ -7628,7 +7637,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="33.75">
+    <row r="14" spans="1:14" ht="34.5">
       <c r="A14" s="61" t="s">
         <v>156</v>
       </c>
@@ -7668,7 +7677,7 @@
       </c>
       <c r="N14" s="10"/>
     </row>
-    <row r="15" spans="1:14" ht="22.5">
+    <row r="15" spans="1:14" ht="23">
       <c r="A15" s="10" t="s">
         <v>159</v>
       </c>
@@ -7710,7 +7719,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="22.5">
+    <row r="16" spans="1:14" ht="23">
       <c r="A16" s="10" t="s">
         <v>162</v>
       </c>
@@ -7752,7 +7761,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="23.25">
+    <row r="17" spans="1:15" ht="23">
       <c r="A17" s="10" t="s">
         <v>166</v>
       </c>
@@ -7796,7 +7805,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="22.5">
+    <row r="18" spans="1:15" ht="23">
       <c r="A18" s="10" t="s">
         <v>171</v>
       </c>
@@ -7878,7 +7887,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="20" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="20" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A20" s="15" t="s">
         <v>177</v>
       </c>
@@ -7921,7 +7930,7 @@
       </c>
       <c r="O20" s="57"/>
     </row>
-    <row r="21" spans="1:15" s="17" customFormat="1" ht="22.5">
+    <row r="21" spans="1:15" s="17" customFormat="1" ht="23">
       <c r="A21" s="15" t="s">
         <v>185</v>
       </c>
@@ -7964,7 +7973,7 @@
       </c>
       <c r="O21" s="83"/>
     </row>
-    <row r="22" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="22" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A22" s="15" t="s">
         <v>190</v>
       </c>
@@ -8007,7 +8016,7 @@
       </c>
       <c r="O22" s="57"/>
     </row>
-    <row r="23" spans="1:15" ht="22.5">
+    <row r="23" spans="1:15" ht="23">
       <c r="A23" s="15" t="s">
         <v>193</v>
       </c>
@@ -8049,7 +8058,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="22.5">
+    <row r="24" spans="1:15" ht="23">
       <c r="A24" s="10" t="s">
         <v>198</v>
       </c>
@@ -8091,7 +8100,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:15" s="18" customFormat="1" ht="22.5">
+    <row r="25" spans="1:15" s="18" customFormat="1" ht="23">
       <c r="A25" s="15" t="s">
         <v>201</v>
       </c>
@@ -8133,7 +8142,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="22.5">
+    <row r="26" spans="1:15" ht="23">
       <c r="A26" s="10" t="s">
         <v>204</v>
       </c>
@@ -8175,7 +8184,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="22.5">
+    <row r="27" spans="1:15" ht="23">
       <c r="A27" s="10" t="s">
         <v>207</v>
       </c>
@@ -8263,7 +8272,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="22.5">
+    <row r="29" spans="1:15" ht="23">
       <c r="A29" s="10" t="s">
         <v>215</v>
       </c>
@@ -8387,7 +8396,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="22.5">
+    <row r="32" spans="1:15" ht="23">
       <c r="A32" s="15" t="s">
         <v>224</v>
       </c>
@@ -8429,7 +8438,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="33" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="33" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A33" s="15" t="s">
         <v>228</v>
       </c>
@@ -8474,7 +8483,7 @@
       </c>
       <c r="O33" s="57"/>
     </row>
-    <row r="34" spans="1:15" ht="22.5">
+    <row r="34" spans="1:15" ht="23">
       <c r="A34" s="10" t="s">
         <v>233</v>
       </c>
@@ -8516,7 +8525,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="15">
+    <row r="35" spans="1:15" ht="14.5">
       <c r="A35" s="10" t="s">
         <v>239</v>
       </c>
@@ -8558,7 +8567,7 @@
       </c>
       <c r="N35" s="10"/>
     </row>
-    <row r="36" spans="1:15" ht="22.5">
+    <row r="36" spans="1:15" ht="23">
       <c r="A36" s="15" t="s">
         <v>243</v>
       </c>
@@ -8642,7 +8651,7 @@
       </c>
       <c r="N37" s="10"/>
     </row>
-    <row r="38" spans="1:15" ht="22.5">
+    <row r="38" spans="1:15" ht="23">
       <c r="A38" s="10" t="s">
         <v>252</v>
       </c>
@@ -8770,7 +8779,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="41" spans="1:15" ht="22.5">
+    <row r="41" spans="1:15" ht="23">
       <c r="A41" s="10" t="s">
         <v>270</v>
       </c>
@@ -8812,7 +8821,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="42" spans="1:15" s="22" customFormat="1" ht="22.5">
+    <row r="42" spans="1:15" s="22" customFormat="1" ht="23">
       <c r="A42" s="10" t="s">
         <v>273</v>
       </c>
@@ -8854,7 +8863,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="43" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="43" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A43" s="15" t="s">
         <v>276</v>
       </c>
@@ -8897,7 +8906,7 @@
       </c>
       <c r="O43" s="57"/>
     </row>
-    <row r="44" spans="1:15" ht="22.5">
+    <row r="44" spans="1:15" ht="23">
       <c r="A44" s="15" t="s">
         <v>281</v>
       </c>
@@ -8939,7 +8948,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="45" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="45" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A45" s="15" t="s">
         <v>284</v>
       </c>
@@ -8982,7 +8991,7 @@
       </c>
       <c r="O45" s="57"/>
     </row>
-    <row r="46" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="46" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A46" s="15" t="s">
         <v>290</v>
       </c>
@@ -9025,7 +9034,7 @@
       </c>
       <c r="O46" s="57"/>
     </row>
-    <row r="47" spans="1:15" ht="22.5">
+    <row r="47" spans="1:15" ht="23">
       <c r="A47" s="10" t="s">
         <v>293</v>
       </c>
@@ -9069,7 +9078,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:15" ht="22.5">
+    <row r="48" spans="1:15" ht="23">
       <c r="A48" s="10" t="s">
         <v>296</v>
       </c>
@@ -9111,7 +9120,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="49" spans="1:15" s="23" customFormat="1" ht="15">
+    <row r="49" spans="1:15" s="23" customFormat="1" ht="14.5">
       <c r="A49" s="24" t="s">
         <v>299</v>
       </c>
@@ -9153,7 +9162,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:15" ht="35.25">
+    <row r="50" spans="1:15" ht="24">
       <c r="A50" s="10" t="s">
         <v>305</v>
       </c>
@@ -9195,7 +9204,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="51" spans="1:15" s="23" customFormat="1" ht="23.25">
+    <row r="51" spans="1:15" s="23" customFormat="1" ht="24">
       <c r="A51" s="24" t="s">
         <v>310</v>
       </c>
@@ -9239,7 +9248,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="52" spans="1:15" ht="22.5">
+    <row r="52" spans="1:15" ht="23">
       <c r="A52" s="10" t="s">
         <v>317</v>
       </c>
@@ -9281,7 +9290,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="53" spans="1:15" ht="23.25">
+    <row r="53" spans="1:15" ht="23">
       <c r="A53" s="10" t="s">
         <v>320</v>
       </c>
@@ -9323,7 +9332,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="54" spans="1:15" ht="22.5">
+    <row r="54" spans="1:15" ht="23">
       <c r="A54" s="10" t="s">
         <v>323</v>
       </c>
@@ -9449,7 +9458,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="57" spans="1:15" s="23" customFormat="1" ht="23.25">
+    <row r="57" spans="1:15" s="23" customFormat="1" ht="24">
       <c r="A57" s="24" t="s">
         <v>333</v>
       </c>
@@ -9493,7 +9502,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="58" spans="1:15" s="23" customFormat="1" ht="23.25">
+    <row r="58" spans="1:15" s="23" customFormat="1" ht="24">
       <c r="A58" s="24" t="s">
         <v>337</v>
       </c>
@@ -9579,7 +9588,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="60" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="60" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A60" s="15" t="s">
         <v>343</v>
       </c>
@@ -9622,7 +9631,7 @@
       </c>
       <c r="O60" s="57"/>
     </row>
-    <row r="61" spans="1:15" ht="22.5">
+    <row r="61" spans="1:15" ht="23">
       <c r="A61" s="10" t="s">
         <v>348</v>
       </c>
@@ -9664,7 +9673,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="62" spans="1:15" ht="22.5">
+    <row r="62" spans="1:15" ht="23">
       <c r="A62" s="10" t="s">
         <v>354</v>
       </c>
@@ -9706,7 +9715,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="63" spans="1:15" s="22" customFormat="1" ht="23.25">
+    <row r="63" spans="1:15" s="22" customFormat="1" ht="23">
       <c r="A63" s="10" t="s">
         <v>357</v>
       </c>
@@ -9958,7 +9967,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="22.5">
+    <row r="69" spans="1:14" ht="23">
       <c r="A69" s="10" t="s">
         <v>380</v>
       </c>
@@ -10000,7 +10009,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="22.5">
+    <row r="70" spans="1:14" ht="23">
       <c r="A70" s="10" t="s">
         <v>384</v>
       </c>
@@ -10042,7 +10051,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="22.5">
+    <row r="71" spans="1:14" ht="23">
       <c r="A71" s="10" t="s">
         <v>387</v>
       </c>
@@ -10084,7 +10093,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="22.5">
+    <row r="72" spans="1:14" ht="23">
       <c r="A72" s="10" t="s">
         <v>391</v>
       </c>
@@ -10168,7 +10177,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="22.5">
+    <row r="74" spans="1:14" ht="23">
       <c r="A74" s="15" t="s">
         <v>397</v>
       </c>
@@ -10212,7 +10221,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="23.25">
+    <row r="75" spans="1:14" ht="23">
       <c r="A75" s="15" t="s">
         <v>403</v>
       </c>
@@ -10254,7 +10263,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="15">
+    <row r="76" spans="1:14" ht="14.5">
       <c r="A76" s="10" t="s">
         <v>406</v>
       </c>
@@ -10294,7 +10303,7 @@
       </c>
       <c r="N76" s="10"/>
     </row>
-    <row r="77" spans="1:14" s="18" customFormat="1" ht="22.5">
+    <row r="77" spans="1:14" s="18" customFormat="1" ht="23">
       <c r="A77" s="31" t="s">
         <v>409</v>
       </c>
@@ -10380,7 +10389,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="79" spans="1:14" s="23" customFormat="1" ht="30">
+    <row r="79" spans="1:14" s="23" customFormat="1" ht="24">
       <c r="A79" s="24" t="s">
         <v>416</v>
       </c>
@@ -10422,7 +10431,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="22.5">
+    <row r="80" spans="1:14" ht="23">
       <c r="A80" s="15" t="s">
         <v>419</v>
       </c>
@@ -10464,7 +10473,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="81" spans="1:15" ht="22.5">
+    <row r="81" spans="1:15" ht="23">
       <c r="A81" s="15" t="s">
         <v>425</v>
       </c>
@@ -10508,7 +10517,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="82" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="82" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A82" s="15" t="s">
         <v>428</v>
       </c>
@@ -10551,7 +10560,7 @@
       </c>
       <c r="O82" s="57"/>
     </row>
-    <row r="83" spans="1:15" s="23" customFormat="1" ht="15">
+    <row r="83" spans="1:15" s="23" customFormat="1" ht="14.5">
       <c r="A83" s="24" t="s">
         <v>432</v>
       </c>
@@ -10593,7 +10602,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="84" spans="1:15" s="23" customFormat="1" ht="15">
+    <row r="84" spans="1:15" s="23" customFormat="1" ht="14.5">
       <c r="A84" s="24" t="s">
         <v>437</v>
       </c>
@@ -10635,7 +10644,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="85" spans="1:15" s="18" customFormat="1" ht="29.25">
+    <row r="85" spans="1:15" s="18" customFormat="1" ht="14.5">
       <c r="A85" s="35" t="s">
         <v>443</v>
       </c>
@@ -10677,7 +10686,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="86" spans="1:15" s="23" customFormat="1" ht="15">
+    <row r="86" spans="1:15" s="23" customFormat="1" ht="14.5">
       <c r="A86" s="24" t="s">
         <v>448</v>
       </c>
@@ -10719,7 +10728,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="87" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="87" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A87" s="15" t="s">
         <v>453</v>
       </c>
@@ -10764,7 +10773,7 @@
       </c>
       <c r="O87" s="57"/>
     </row>
-    <row r="88" spans="1:15" s="42" customFormat="1" ht="22.5">
+    <row r="88" spans="1:15" s="42" customFormat="1" ht="23">
       <c r="A88" s="31" t="s">
         <v>458</v>
       </c>
@@ -10809,7 +10818,7 @@
       </c>
       <c r="O88" s="84"/>
     </row>
-    <row r="89" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="89" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A89" s="15" t="s">
         <v>461</v>
       </c>
@@ -10852,7 +10861,7 @@
       </c>
       <c r="O89" s="57"/>
     </row>
-    <row r="90" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="90" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A90" s="15" t="s">
         <v>466</v>
       </c>
@@ -10895,7 +10904,7 @@
       </c>
       <c r="O90" s="57"/>
     </row>
-    <row r="91" spans="1:15" ht="22.5">
+    <row r="91" spans="1:15" ht="23">
       <c r="A91" s="10" t="s">
         <v>469</v>
       </c>
@@ -10937,7 +10946,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="92" spans="1:15" ht="22.5">
+    <row r="92" spans="1:15" ht="23">
       <c r="A92" s="15" t="s">
         <v>472</v>
       </c>
@@ -11021,7 +11030,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="94" spans="1:15" s="18" customFormat="1" ht="15">
+    <row r="94" spans="1:15" s="18" customFormat="1" ht="14.5">
       <c r="A94" s="35" t="s">
         <v>479</v>
       </c>
@@ -11097,7 +11106,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="96" spans="1:15" ht="22.5">
+    <row r="96" spans="1:15" ht="23">
       <c r="A96" s="10" t="s">
         <v>485</v>
       </c>
@@ -11139,7 +11148,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="97" spans="1:15" ht="22.5">
+    <row r="97" spans="1:15" ht="23">
       <c r="A97" s="15" t="s">
         <v>488</v>
       </c>
@@ -11181,7 +11190,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="98" spans="1:15" ht="22.5">
+    <row r="98" spans="1:15" ht="23">
       <c r="A98" s="15" t="s">
         <v>491</v>
       </c>
@@ -11223,7 +11232,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="99" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="99" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A99" s="15" t="s">
         <v>496</v>
       </c>
@@ -11266,7 +11275,7 @@
       </c>
       <c r="O99" s="57"/>
     </row>
-    <row r="100" spans="1:15" ht="23.25">
+    <row r="100" spans="1:15" ht="23">
       <c r="A100" s="10" t="s">
         <v>500</v>
       </c>
@@ -11350,7 +11359,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="102" spans="1:15" ht="22.5">
+    <row r="102" spans="1:15" ht="23">
       <c r="A102" s="10" t="s">
         <v>507</v>
       </c>
@@ -11434,7 +11443,7 @@
       </c>
       <c r="N103" s="10"/>
     </row>
-    <row r="104" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="104" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A104" s="15" t="s">
         <v>513</v>
       </c>
@@ -11477,7 +11486,7 @@
       </c>
       <c r="O104" s="57"/>
     </row>
-    <row r="105" spans="1:15" ht="22.5">
+    <row r="105" spans="1:15" ht="23">
       <c r="A105" s="10" t="s">
         <v>518</v>
       </c>
@@ -11519,7 +11528,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="106" spans="1:15" s="16" customFormat="1" ht="22.5">
+    <row r="106" spans="1:15" s="16" customFormat="1" ht="23">
       <c r="A106" s="15" t="s">
         <v>523</v>
       </c>
@@ -11562,7 +11571,7 @@
       </c>
       <c r="O106" s="57"/>
     </row>
-    <row r="107" spans="1:15" ht="22.5">
+    <row r="107" spans="1:15" ht="23">
       <c r="A107" s="15" t="s">
         <v>526</v>
       </c>
@@ -11604,7 +11613,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="108" spans="1:15" ht="22.5">
+    <row r="108" spans="1:15" ht="23">
       <c r="A108" s="10" t="s">
         <v>529</v>
       </c>
@@ -11690,7 +11699,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="110" spans="1:15" s="23" customFormat="1" ht="23.25">
+    <row r="110" spans="1:15" s="23" customFormat="1" ht="24">
       <c r="A110" s="24" t="s">
         <v>535</v>
       </c>
@@ -11816,7 +11825,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="113" spans="1:14" s="18" customFormat="1" ht="22.5">
+    <row r="113" spans="1:14" s="18" customFormat="1" ht="23">
       <c r="A113" s="10" t="s">
         <v>544</v>
       </c>
@@ -11902,7 +11911,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="115" spans="1:14" ht="22.5">
+    <row r="115" spans="1:14" ht="23">
       <c r="A115" s="10" t="s">
         <v>550</v>
       </c>
@@ -11986,7 +11995,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="117" spans="1:14" ht="22.5">
+    <row r="117" spans="1:14" ht="23">
       <c r="A117" s="15" t="s">
         <v>556</v>
       </c>
@@ -12028,7 +12037,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="118" spans="1:14" s="18" customFormat="1" ht="15">
+    <row r="118" spans="1:14" s="18" customFormat="1" ht="14.5">
       <c r="A118" s="35" t="s">
         <v>559</v>
       </c>
@@ -12070,7 +12079,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="119" spans="1:14" s="18" customFormat="1" ht="15">
+    <row r="119" spans="1:14" s="18" customFormat="1" ht="14.5">
       <c r="A119" s="35" t="s">
         <v>562</v>
       </c>
@@ -12112,7 +12121,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="120" spans="1:14" ht="22.5">
+    <row r="120" spans="1:14" ht="23">
       <c r="A120" s="10" t="s">
         <v>565</v>
       </c>
@@ -12154,7 +12163,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="121" spans="1:14" ht="22.5">
+    <row r="121" spans="1:14" ht="23">
       <c r="A121" s="10" t="s">
         <v>568</v>
       </c>
@@ -12196,7 +12205,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="122" spans="1:14" ht="22.5">
+    <row r="122" spans="1:14" ht="23">
       <c r="A122" s="10" t="s">
         <v>571</v>
       </c>
@@ -12238,7 +12247,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="123" spans="1:14" ht="22.5">
+    <row r="123" spans="1:14" ht="23">
       <c r="A123" s="10" t="s">
         <v>574</v>
       </c>
@@ -12282,7 +12291,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="124" spans="1:14" s="8" customFormat="1" ht="33.75">
+    <row r="124" spans="1:14" s="8" customFormat="1" ht="34.5">
       <c r="A124" s="10" t="s">
         <v>577</v>
       </c>
@@ -12324,7 +12333,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="125" spans="1:14" ht="22.5">
+    <row r="125" spans="1:14" ht="23">
       <c r="A125" s="10" t="s">
         <v>582</v>
       </c>
@@ -12366,7 +12375,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="126" spans="1:14" ht="22.5">
+    <row r="126" spans="1:14" ht="23">
       <c r="A126" s="15" t="s">
         <v>585</v>
       </c>
@@ -12408,7 +12417,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="127" spans="1:14" s="18" customFormat="1" ht="22.5">
+    <row r="127" spans="1:14" s="18" customFormat="1" ht="23">
       <c r="A127" s="35" t="s">
         <v>588</v>
       </c>
@@ -12450,7 +12459,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="128" spans="1:14" s="23" customFormat="1" ht="15">
+    <row r="128" spans="1:14" s="23" customFormat="1" ht="14.5">
       <c r="A128" s="24" t="s">
         <v>591</v>
       </c>
@@ -12490,7 +12499,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="129" spans="1:15" ht="23.25">
+    <row r="129" spans="1:15" ht="23">
       <c r="A129" s="10" t="s">
         <v>594</v>
       </c>
@@ -12534,7 +12543,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="130" spans="1:15" s="45" customFormat="1" ht="22.5">
+    <row r="130" spans="1:15" s="45" customFormat="1" ht="23">
       <c r="A130" s="31" t="s">
         <v>597</v>
       </c>
@@ -12577,7 +12586,7 @@
       </c>
       <c r="O130" s="85"/>
     </row>
-    <row r="131" spans="1:15" ht="23.25">
+    <row r="131" spans="1:15" ht="23">
       <c r="A131" s="10" t="s">
         <v>600</v>
       </c>
@@ -12621,7 +12630,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="132" spans="1:15" s="46" customFormat="1" ht="22.5">
+    <row r="132" spans="1:15" s="46" customFormat="1" ht="23">
       <c r="A132" s="35" t="s">
         <v>603</v>
       </c>
@@ -12663,7 +12672,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="133" spans="1:15" ht="22.5">
+    <row r="133" spans="1:15" ht="23">
       <c r="A133" s="15" t="s">
         <v>606</v>
       </c>
@@ -12705,7 +12714,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="134" spans="1:15" s="45" customFormat="1" ht="22.5">
+    <row r="134" spans="1:15" s="45" customFormat="1" ht="23">
       <c r="A134" s="31" t="s">
         <v>609</v>
       </c>
@@ -12748,7 +12757,7 @@
       </c>
       <c r="O134" s="85"/>
     </row>
-    <row r="135" spans="1:15" s="18" customFormat="1" ht="15">
+    <row r="135" spans="1:15" s="18" customFormat="1" ht="14.5">
       <c r="A135" s="31" t="s">
         <v>612</v>
       </c>
@@ -12786,7 +12795,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="136" spans="1:15" ht="15">
+    <row r="136" spans="1:15" ht="14.5">
       <c r="A136" s="47"/>
       <c r="B136" s="48"/>
       <c r="C136" s="47"/>
@@ -12833,10 +12842,10 @@
       <c r="M138" s="47"/>
       <c r="N138" s="47"/>
     </row>
-    <row r="139" spans="1:15" ht="15.75">
+    <row r="139" spans="1:15" ht="16">
       <c r="L139" s="60"/>
     </row>
-    <row r="140" spans="1:15" ht="15.75">
+    <row r="140" spans="1:15" ht="16">
       <c r="L140" s="60"/>
     </row>
     <row r="141" spans="1:15">
@@ -12856,28 +12865,28 @@
   <conditionalFormatting sqref="G37">
     <cfRule type="duplicateValues" dxfId="7" priority="7"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G49">
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G51">
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G57">
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G58">
+    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G103">
-    <cfRule type="duplicateValues" dxfId="6" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G118">
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L143:L65509">
-    <cfRule type="expression" dxfId="5" priority="95" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="95" stopIfTrue="1">
       <formula>AND(COUNTIF($L$131:$L$65509, L143)+COUNTIF($L$2:$L$2, L143)&gt;1,NOT(ISBLANK(L143)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G49">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G118">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G58">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G51">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G57">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="75" orientation="landscape" verticalDpi="599" r:id="rId1"/>
@@ -12885,15 +12894,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <SharedWithUsers xmlns="1ca80d59-04e9-4dec-91ac-1ecebfe0c492">
@@ -12905,6 +12905,15 @@
     </SharedWithUsers>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13085,13 +13094,38 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FAC3CCFC-5F0F-4431-BF21-C2397D0A3104}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557D19C1-22A9-4FF4-AAF0-C925D251FEE7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1ca80d59-04e9-4dec-91ac-1ecebfe0c492"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557D19C1-22A9-4FF4-AAF0-C925D251FEE7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FAC3CCFC-5F0F-4431-BF21-C2397D0A3104}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE734FC9-2FB2-4410-B63B-9C01F7B74935}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE734FC9-2FB2-4410-B63B-9C01F7B74935}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="425754f6-b54f-4cc4-9c19-ccb7c8d18432"/>
+    <ds:schemaRef ds:uri="1ca80d59-04e9-4dec-91ac-1ecebfe0c492"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>